<commit_message>
feat: shacls sereiesMember and rightsStatement
added shacls for seriesMember and extended rightsStatement class
</commit_message>
<xml_diff>
--- a/Formalisation(shacl)/Core/SHACL_pipeline_templates/SHACL-dataset.xlsx
+++ b/Formalisation(shacl)/Core/SHACL_pipeline_templates/SHACL-dataset.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://healthri.sharepoint.com/sites/hri-team012/Shared Documents/A-Team/26 - Implementation/50 - Technical/V2 Shapes/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://healthri-my.sharepoint.com/personal/hannah_neikes_health-ri_nl/Documents/Documenten/GitHub/health-ri-metadata/Formalisation(shacl)/Core/SHACL_pipeline_templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="282" documentId="13_ncr:1_{1B1DBC4C-3AF0-9940-9D98-49079FB71514}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F226E0A5-FBB4-A74C-AD48-2FABBA4A1AA4}"/>
+  <xr:revisionPtr revIDLastSave="283" documentId="13_ncr:1_{1B1DBC4C-3AF0-9940-9D98-49079FB71514}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{58F2A9B4-EA8E-453C-9FFC-DC61F2DAD80F}"/>
   <bookViews>
-    <workbookView xWindow="-17820" yWindow="-28300" windowWidth="36000" windowHeight="22500" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30612" yWindow="-12576" windowWidth="30936" windowHeight="16776" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="prefixes" sheetId="1" r:id="rId1"/>
@@ -2003,7 +2003,6 @@
     <cellStyle name="Neutre 2 2" xfId="126" xr:uid="{00000000-0005-0000-0000-000083000000}"/>
     <cellStyle name="Neutre 3" xfId="127" xr:uid="{00000000-0005-0000-0000-000084000000}"/>
     <cellStyle name="Neutre 3 2" xfId="128" xr:uid="{00000000-0005-0000-0000-000085000000}"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 10" xfId="129" xr:uid="{00000000-0005-0000-0000-000086000000}"/>
     <cellStyle name="Normal 2" xfId="130" xr:uid="{00000000-0005-0000-0000-000087000000}"/>
     <cellStyle name="Normal 2 2" xfId="131" xr:uid="{00000000-0005-0000-0000-000088000000}"/>
@@ -2030,6 +2029,7 @@
     <cellStyle name="Normal 9 3" xfId="152" xr:uid="{00000000-0005-0000-0000-00009D000000}"/>
     <cellStyle name="Note 17" xfId="153" xr:uid="{00000000-0005-0000-0000-00009E000000}"/>
     <cellStyle name="Result (user) 18" xfId="154" xr:uid="{00000000-0005-0000-0000-00009F000000}"/>
+    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
     <cellStyle name="Status 19" xfId="155" xr:uid="{00000000-0005-0000-0000-0000A0000000}"/>
     <cellStyle name="Text 20" xfId="156" xr:uid="{00000000-0005-0000-0000-0000A1000000}"/>
     <cellStyle name="Titre 2" xfId="157" xr:uid="{00000000-0005-0000-0000-0000A2000000}"/>
@@ -2225,13 +2225,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A2:C26"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="10.77734375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="19" customWidth="1"/>
-    <col min="3" max="3" width="59.5" customWidth="1"/>
+    <col min="3" max="3" width="59.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -2242,7 +2242,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -2253,7 +2253,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>0</v>
       </c>
@@ -2264,7 +2264,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>0</v>
       </c>
@@ -2275,7 +2275,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>0</v>
       </c>
@@ -2286,7 +2286,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>0</v>
       </c>
@@ -2297,7 +2297,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>0</v>
       </c>
@@ -2308,7 +2308,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>0</v>
       </c>
@@ -2319,7 +2319,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>0</v>
       </c>
@@ -2330,7 +2330,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>0</v>
       </c>
@@ -2341,7 +2341,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>0</v>
       </c>
@@ -2352,7 +2352,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>0</v>
       </c>
@@ -2363,7 +2363,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>0</v>
       </c>
@@ -2374,7 +2374,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>0</v>
       </c>
@@ -2385,7 +2385,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="56" t="s">
         <v>0</v>
       </c>
@@ -2396,7 +2396,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>0</v>
       </c>
@@ -2407,7 +2407,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>0</v>
       </c>
@@ -2418,7 +2418,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>0</v>
       </c>
@@ -2429,7 +2429,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>0</v>
       </c>
@@ -2440,7 +2440,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>0</v>
       </c>
@@ -2451,7 +2451,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>0</v>
       </c>
@@ -2462,7 +2462,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>0</v>
       </c>
@@ -2473,7 +2473,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>0</v>
       </c>
@@ -2484,7 +2484,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>0</v>
       </c>
@@ -2495,7 +2495,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>0</v>
       </c>
@@ -2536,24 +2536,24 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:M15"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.5" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="8.44140625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="27.83203125" customWidth="1"/>
-    <col min="2" max="2" width="30.83203125" customWidth="1"/>
+    <col min="1" max="1" width="27.77734375" customWidth="1"/>
+    <col min="2" max="2" width="30.77734375" customWidth="1"/>
     <col min="3" max="3" width="42.33203125" customWidth="1"/>
-    <col min="4" max="5" width="38.83203125" customWidth="1"/>
-    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+    <col min="4" max="5" width="38.77734375" customWidth="1"/>
+    <col min="6" max="6" width="18.77734375" customWidth="1"/>
     <col min="7" max="7" width="25.33203125" style="5" customWidth="1"/>
     <col min="8" max="8" width="16.33203125" style="5" customWidth="1"/>
-    <col min="9" max="9" width="31.1640625" style="5" customWidth="1"/>
+    <col min="9" max="9" width="31.109375" style="5" customWidth="1"/>
     <col min="10" max="10" width="52" customWidth="1"/>
     <col min="11" max="11" width="40" style="5" customWidth="1"/>
-    <col min="12" max="12" width="20.5" customWidth="1"/>
+    <col min="12" max="12" width="20.44140625" customWidth="1"/>
     <col min="13" max="13" width="27.33203125" customWidth="1"/>
-    <col min="1014" max="1018" width="11.5" customWidth="1"/>
+    <col min="1014" max="1018" width="11.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>51</v>
       </c>
@@ -2562,7 +2562,7 @@
       </c>
       <c r="F1" s="3"/>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>52</v>
       </c>
@@ -2571,7 +2571,7 @@
       </c>
       <c r="F2" s="3"/>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>54</v>
       </c>
@@ -2580,7 +2580,7 @@
       </c>
       <c r="F3" s="3"/>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>56</v>
       </c>
@@ -2589,7 +2589,7 @@
       </c>
       <c r="F4" s="3"/>
     </row>
-    <row r="5" spans="1:13" ht="28" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:13" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>57</v>
       </c>
@@ -2598,7 +2598,7 @@
       </c>
       <c r="F5" s="3"/>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>59</v>
       </c>
@@ -2607,7 +2607,7 @@
       </c>
       <c r="F6" s="3"/>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>61</v>
       </c>
@@ -2616,10 +2616,10 @@
       </c>
       <c r="F7" s="3"/>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="G8" s="7"/>
     </row>
-    <row r="9" spans="1:13" s="8" customFormat="1" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
         <v>62</v>
       </c>
@@ -2628,7 +2628,7 @@
       <c r="I9" s="11"/>
       <c r="K9" s="11"/>
     </row>
-    <row r="10" spans="1:13" s="8" customFormat="1" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
         <v>63</v>
       </c>
@@ -2640,7 +2640,7 @@
       <c r="I10" s="11"/>
       <c r="K10" s="11"/>
     </row>
-    <row r="12" spans="1:13" s="13" customFormat="1" ht="89.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:13" s="13" customFormat="1" ht="89.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
         <v>65</v>
       </c>
@@ -2681,7 +2681,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="44.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:13" ht="44.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="17" t="s">
         <v>78</v>
       </c>
@@ -2722,7 +2722,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="14" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="57" t="s">
         <v>89</v>
       </c>
@@ -2739,7 +2739,7 @@
       <c r="K14" s="21"/>
       <c r="M14" s="22"/>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="5"/>
       <c r="B15" s="5"/>
       <c r="D15" s="5"/>
@@ -2767,32 +2767,32 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:X60"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="38.5" customWidth="1"/>
-    <col min="2" max="2" width="41.5" style="5" customWidth="1"/>
+    <col min="1" max="1" width="38.44140625" customWidth="1"/>
+    <col min="2" max="2" width="41.44140625" style="5" customWidth="1"/>
     <col min="3" max="3" width="42.6640625" customWidth="1"/>
-    <col min="4" max="4" width="26.83203125" style="23" customWidth="1"/>
-    <col min="5" max="5" width="41.5" style="5" customWidth="1"/>
+    <col min="4" max="4" width="26.77734375" style="23" customWidth="1"/>
+    <col min="5" max="5" width="41.44140625" style="5" customWidth="1"/>
     <col min="6" max="6" width="31.33203125" style="22" customWidth="1"/>
-    <col min="7" max="7" width="14.5" style="24" customWidth="1"/>
+    <col min="7" max="7" width="14.44140625" style="24" customWidth="1"/>
     <col min="8" max="8" width="12" style="25" customWidth="1"/>
-    <col min="9" max="9" width="20.1640625" customWidth="1"/>
+    <col min="9" max="9" width="20.109375" customWidth="1"/>
     <col min="10" max="10" width="21" customWidth="1"/>
     <col min="11" max="11" width="18" customWidth="1"/>
     <col min="12" max="14" width="26" hidden="1" customWidth="1"/>
-    <col min="15" max="15" width="17.5" customWidth="1"/>
+    <col min="15" max="15" width="17.44140625" customWidth="1"/>
     <col min="16" max="16" width="36" hidden="1" customWidth="1"/>
-    <col min="17" max="17" width="34.83203125" hidden="1" customWidth="1"/>
-    <col min="18" max="18" width="17.83203125" customWidth="1"/>
+    <col min="17" max="17" width="34.77734375" hidden="1" customWidth="1"/>
+    <col min="18" max="18" width="17.77734375" customWidth="1"/>
     <col min="19" max="19" width="14.6640625" style="5" customWidth="1"/>
     <col min="20" max="22" width="15.6640625" style="5" customWidth="1"/>
-    <col min="23" max="23" width="17.1640625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="24.1640625" bestFit="1" customWidth="1"/>
-    <col min="1021" max="1025" width="11.5" customWidth="1"/>
+    <col min="23" max="23" width="17.109375" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="24.109375" bestFit="1" customWidth="1"/>
+    <col min="1021" max="1025" width="11.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="13" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:24" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>51</v>
       </c>
@@ -2803,7 +2803,7 @@
       <c r="O1" s="5"/>
       <c r="R1" s="5"/>
     </row>
-    <row r="3" spans="1:24" s="8" customFormat="1" ht="13" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:24" s="8" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>93</v>
       </c>
@@ -2819,12 +2819,12 @@
       <c r="U3" s="11"/>
       <c r="V3" s="11"/>
     </row>
-    <row r="4" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D4" s="29"/>
       <c r="G4" s="30"/>
       <c r="P4" s="5"/>
     </row>
-    <row r="5" spans="1:24" s="14" customFormat="1" ht="112" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:24" s="14" customFormat="1" ht="105.6" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>94</v>
       </c>
@@ -2886,7 +2886,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="6" spans="1:24" s="33" customFormat="1" ht="28" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:24" s="33" customFormat="1" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A6" s="33" t="s">
         <v>114</v>
       </c>
@@ -2908,7 +2908,7 @@
       <c r="G6" s="36"/>
       <c r="H6" s="36"/>
     </row>
-    <row r="7" spans="1:24" ht="42" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:24" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A7" s="37" t="s">
         <v>78</v>
       </c>
@@ -2982,7 +2982,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="8" spans="1:24" s="42" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:24" s="42" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="42" t="s">
         <v>140</v>
       </c>
@@ -2996,7 +2996,7 @@
       <c r="U8" s="46"/>
       <c r="V8" s="46"/>
     </row>
-    <row r="9" spans="1:24" ht="64" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:24" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A9" s="47" t="str">
         <f t="shared" ref="A9:A55" si="0">CONCATENATE(B9,"#",SUBSTITUTE(D9," ","-"))</f>
         <v>hri:DatasetShape#access-rights</v>
@@ -3032,7 +3032,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="10" spans="1:24" ht="16" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:24" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A10" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#analytics</v>
@@ -3060,7 +3060,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="11" spans="1:24" ht="48" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:24" ht="43.2" x14ac:dyDescent="0.25">
       <c r="A11" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#applicable-legislation</v>
@@ -3093,7 +3093,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="12" spans="1:24" ht="32" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:24" ht="28.8" x14ac:dyDescent="0.25">
       <c r="A12" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#code-values</v>
@@ -3121,7 +3121,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="13" spans="1:24" ht="32" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:24" ht="28.8" x14ac:dyDescent="0.25">
       <c r="A13" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#coding-system</v>
@@ -3149,7 +3149,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="14" spans="1:24" ht="16" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:24" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A14" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#conforms-to</v>
@@ -3177,7 +3177,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="15" spans="1:24" ht="32" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:24" ht="28.8" x14ac:dyDescent="0.25">
       <c r="A15" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#contact-point</v>
@@ -3205,13 +3205,13 @@
         <v>168</v>
       </c>
       <c r="W15" s="56" t="s">
-        <v>146</v>
+        <v>174</v>
       </c>
       <c r="X15" s="56" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="16" spans="1:24" ht="16" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:24" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A16" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#creator</v>
@@ -3242,7 +3242,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="17" spans="1:24" ht="16" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:24" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A17" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#description</v>
@@ -3276,7 +3276,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="18" spans="1:24" ht="16" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:24" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A18" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#distribution</v>
@@ -3304,7 +3304,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="19" spans="1:24" ht="16" x14ac:dyDescent="0.15">
+    <row r="19" spans="1:24" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A19" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#documentation</v>
@@ -3332,7 +3332,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="20" spans="1:24" ht="48" x14ac:dyDescent="0.15">
+    <row r="20" spans="1:24" ht="43.2" x14ac:dyDescent="0.25">
       <c r="A20" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#frequency</v>
@@ -3364,7 +3364,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="21" spans="1:24" ht="50.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:24" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#geographical-coverage</v>
@@ -3392,7 +3392,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="22" spans="1:24" ht="37.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="22" spans="1:24" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#has-version</v>
@@ -3420,7 +3420,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="23" spans="1:24" ht="29.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="23" spans="1:24" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#health-theme</v>
@@ -3448,7 +3448,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="24" spans="1:24" ht="14" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="24" spans="1:24" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#identifier</v>
@@ -3482,7 +3482,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="25" spans="1:24" ht="16" x14ac:dyDescent="0.15">
+    <row r="25" spans="1:24" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A25" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#in-series</v>
@@ -3510,7 +3510,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="26" spans="1:24" ht="32" x14ac:dyDescent="0.15">
+    <row r="26" spans="1:24" ht="43.2" x14ac:dyDescent="0.25">
       <c r="A26" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#is-referenced-by</v>
@@ -3538,7 +3538,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="27" spans="1:24" ht="16" x14ac:dyDescent="0.15">
+    <row r="27" spans="1:24" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A27" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#keyword</v>
@@ -3569,7 +3569,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="28" spans="1:24" ht="32" x14ac:dyDescent="0.15">
+    <row r="28" spans="1:24" ht="28.8" x14ac:dyDescent="0.25">
       <c r="A28" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#language</v>
@@ -3597,7 +3597,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="29" spans="1:24" ht="64" x14ac:dyDescent="0.15">
+    <row r="29" spans="1:24" ht="72" x14ac:dyDescent="0.25">
       <c r="A29" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#legal-basis</v>
@@ -3625,7 +3625,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="30" spans="1:24" ht="32" x14ac:dyDescent="0.15">
+    <row r="30" spans="1:24" ht="28.8" x14ac:dyDescent="0.25">
       <c r="A30" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#maximum-typical-age</v>
@@ -3659,7 +3659,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="31" spans="1:24" ht="32" x14ac:dyDescent="0.15">
+    <row r="31" spans="1:24" ht="28.8" x14ac:dyDescent="0.25">
       <c r="A31" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#minimum-typical-age</v>
@@ -3693,7 +3693,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="32" spans="1:24" ht="32" x14ac:dyDescent="0.15">
+    <row r="32" spans="1:24" ht="28.8" x14ac:dyDescent="0.25">
       <c r="A32" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#modification-date</v>
@@ -3730,7 +3730,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="33" spans="1:24" ht="16" x14ac:dyDescent="0.15">
+    <row r="33" spans="1:24" ht="28.8" x14ac:dyDescent="0.25">
       <c r="A33" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#number-of-records</v>
@@ -3764,7 +3764,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="34" spans="1:24" ht="16" x14ac:dyDescent="0.15">
+    <row r="34" spans="1:24" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A34" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#number-of-unique-infividuals</v>
@@ -3798,7 +3798,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="35" spans="1:24" ht="48" x14ac:dyDescent="0.15">
+    <row r="35" spans="1:24" ht="43.2" x14ac:dyDescent="0.25">
       <c r="A35" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#other-identifier</v>
@@ -3827,7 +3827,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="36" spans="1:24" ht="48" x14ac:dyDescent="0.15">
+    <row r="36" spans="1:24" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A36" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#personal-data</v>
@@ -3855,7 +3855,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="37" spans="1:24" ht="16" x14ac:dyDescent="0.15">
+    <row r="37" spans="1:24" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A37" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#population-coverage</v>
@@ -3884,7 +3884,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="38" spans="1:24" ht="32" x14ac:dyDescent="0.15">
+    <row r="38" spans="1:24" ht="28.8" x14ac:dyDescent="0.25">
       <c r="A38" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#publisher</v>
@@ -3918,7 +3918,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="39" spans="1:24" ht="80" x14ac:dyDescent="0.15">
+    <row r="39" spans="1:24" ht="72" x14ac:dyDescent="0.25">
       <c r="A39" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#purpose</v>
@@ -3946,7 +3946,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="40" spans="1:24" ht="32" x14ac:dyDescent="0.15">
+    <row r="40" spans="1:24" ht="28.8" x14ac:dyDescent="0.25">
       <c r="A40" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#qualified-attribution</v>
@@ -3975,7 +3975,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="41" spans="1:24" ht="16" x14ac:dyDescent="0.15">
+    <row r="41" spans="1:24" ht="28.8" x14ac:dyDescent="0.25">
       <c r="A41" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#qualified-relation</v>
@@ -4004,7 +4004,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="42" spans="1:24" ht="48" x14ac:dyDescent="0.15">
+    <row r="42" spans="1:24" ht="43.2" x14ac:dyDescent="0.25">
       <c r="A42" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#quality-annotation</v>
@@ -4033,7 +4033,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="43" spans="1:24" ht="32" x14ac:dyDescent="0.15">
+    <row r="43" spans="1:24" ht="28.8" x14ac:dyDescent="0.25">
       <c r="A43" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#release-date</v>
@@ -4070,7 +4070,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="44" spans="1:24" ht="32" x14ac:dyDescent="0.15">
+    <row r="44" spans="1:24" ht="28.8" x14ac:dyDescent="0.25">
       <c r="A44" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#retention-period</v>
@@ -4102,7 +4102,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="45" spans="1:24" ht="16" x14ac:dyDescent="0.15">
+    <row r="45" spans="1:24" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A45" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#sample</v>
@@ -4130,7 +4130,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="46" spans="1:24" ht="32" x14ac:dyDescent="0.15">
+    <row r="46" spans="1:24" ht="28.8" x14ac:dyDescent="0.25">
       <c r="A46" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#source</v>
@@ -4158,7 +4158,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="47" spans="1:24" ht="32" x14ac:dyDescent="0.15">
+    <row r="47" spans="1:24" ht="28.8" x14ac:dyDescent="0.25">
       <c r="A47" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#status</v>
@@ -4189,7 +4189,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="48" spans="1:24" ht="16" x14ac:dyDescent="0.15">
+    <row r="48" spans="1:24" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A48" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#temporal-coverage</v>
@@ -4218,7 +4218,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="49" spans="1:24" ht="16" x14ac:dyDescent="0.15">
+    <row r="49" spans="1:24" ht="28.8" x14ac:dyDescent="0.25">
       <c r="A49" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#temporal-resolution</v>
@@ -4252,7 +4252,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="50" spans="1:24" ht="80" x14ac:dyDescent="0.15">
+    <row r="50" spans="1:24" ht="72" x14ac:dyDescent="0.25">
       <c r="A50" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#theme</v>
@@ -4285,7 +4285,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="51" spans="1:24" ht="16" x14ac:dyDescent="0.15">
+    <row r="51" spans="1:24" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A51" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#title</v>
@@ -4319,7 +4319,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="52" spans="1:24" ht="32" x14ac:dyDescent="0.15">
+    <row r="52" spans="1:24" ht="28.8" x14ac:dyDescent="0.25">
       <c r="A52" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#type</v>
@@ -4347,7 +4347,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="53" spans="1:24" ht="16" x14ac:dyDescent="0.15">
+    <row r="53" spans="1:24" ht="28.8" x14ac:dyDescent="0.25">
       <c r="A53" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#version</v>
@@ -4379,7 +4379,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="54" spans="1:24" ht="32" x14ac:dyDescent="0.15">
+    <row r="54" spans="1:24" ht="28.8" x14ac:dyDescent="0.25">
       <c r="A54" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#version-notes</v>
@@ -4411,7 +4411,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="55" spans="1:24" ht="32" x14ac:dyDescent="0.15">
+    <row r="55" spans="1:24" ht="28.8" x14ac:dyDescent="0.25">
       <c r="A55" s="47" t="str">
         <f t="shared" si="0"/>
         <v>hri:DatasetShape#was-generated-by</v>
@@ -4439,7 +4439,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="56" spans="1:24" s="58" customFormat="1" ht="15" x14ac:dyDescent="0.15">
+    <row r="56" spans="1:24" s="58" customFormat="1" ht="14.4" x14ac:dyDescent="0.25">
       <c r="B56" s="59"/>
       <c r="C56" s="60"/>
       <c r="D56" s="60"/>
@@ -4455,7 +4455,7 @@
       <c r="W56" s="65"/>
       <c r="X56" s="65"/>
     </row>
-    <row r="57" spans="1:24" s="58" customFormat="1" ht="13" x14ac:dyDescent="0.15">
+    <row r="57" spans="1:24" s="58" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
       <c r="B57" s="59"/>
       <c r="D57" s="66"/>
       <c r="E57" s="61"/>
@@ -4467,7 +4467,7 @@
       <c r="U57" s="61"/>
       <c r="V57" s="61"/>
     </row>
-    <row r="58" spans="1:24" s="58" customFormat="1" ht="13" x14ac:dyDescent="0.15">
+    <row r="58" spans="1:24" s="58" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
       <c r="B58" s="59"/>
       <c r="D58" s="66"/>
       <c r="E58" s="61"/>
@@ -4479,7 +4479,7 @@
       <c r="U58" s="61"/>
       <c r="V58" s="61"/>
     </row>
-    <row r="59" spans="1:24" s="58" customFormat="1" ht="13" x14ac:dyDescent="0.15">
+    <row r="59" spans="1:24" s="58" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
       <c r="B59" s="59"/>
       <c r="D59" s="66"/>
       <c r="E59" s="61"/>
@@ -4491,7 +4491,7 @@
       <c r="U59" s="61"/>
       <c r="V59" s="61"/>
     </row>
-    <row r="60" spans="1:24" s="58" customFormat="1" ht="13" x14ac:dyDescent="0.15">
+    <row r="60" spans="1:24" s="58" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
       <c r="B60" s="59"/>
       <c r="D60" s="66"/>
       <c r="E60" s="61"/>
@@ -4524,6 +4524,36 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="cfc87205-1831-4b6c-a7b4-76d40079a43e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="221af607-abea-4d5e-830c-567dcc03c0ec" xsi:nil="true"/>
+    <Categorie xmlns="cfc87205-1831-4b6c-a7b4-76d40079a43e" xsi:nil="true"/>
+    <_Flow_SignoffStatus xmlns="cfc87205-1831-4b6c-a7b4-76d40079a43e" xsi:nil="true"/>
+    <Persoon xmlns="cfc87205-1831-4b6c-a7b4-76d40079a43e">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Persoon>
+    <Opmerkingen xmlns="cfc87205-1831-4b6c-a7b4-76d40079a43e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000B1A1CF98C819F4881BB4349588D0C85" ma:contentTypeVersion="22" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="31f6c59cfd598d1d7de5b45c1822abcd">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="cfc87205-1831-4b6c-a7b4-76d40079a43e" xmlns:ns3="221af607-abea-4d5e-830c-567dcc03c0ec" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="67714481eaab3d0eef8b708c465ce66d" ns2:_="" ns3:_="">
     <xsd:import namespace="cfc87205-1831-4b6c-a7b4-76d40079a43e"/>
@@ -4811,37 +4841,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D188C3D5-44E3-4A45-B4C8-A1EF171C14AD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="221af607-abea-4d5e-830c-567dcc03c0ec"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="cfc87205-1831-4b6c-a7b4-76d40079a43e"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="cfc87205-1831-4b6c-a7b4-76d40079a43e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="221af607-abea-4d5e-830c-567dcc03c0ec" xsi:nil="true"/>
-    <Categorie xmlns="cfc87205-1831-4b6c-a7b4-76d40079a43e" xsi:nil="true"/>
-    <_Flow_SignoffStatus xmlns="cfc87205-1831-4b6c-a7b4-76d40079a43e" xsi:nil="true"/>
-    <Persoon xmlns="cfc87205-1831-4b6c-a7b4-76d40079a43e">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Persoon>
-    <Opmerkingen xmlns="cfc87205-1831-4b6c-a7b4-76d40079a43e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{714965F3-B175-40D4-A6BA-6E5740C5D9B2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DEF8A8EB-FDDC-4F03-BB17-434FEEA9C2D7}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4858,29 +4883,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{714965F3-B175-40D4-A6BA-6E5740C5D9B2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D188C3D5-44E3-4A45-B4C8-A1EF171C14AD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="221af607-abea-4d5e-830c-567dcc03c0ec"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="cfc87205-1831-4b6c-a7b4-76d40079a43e"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>